<commit_message>
chore: dae_il/graphy 결과 업데이트 + data_injector 대상 시트 자동 생성 처리
- data_injector.py: 대상 시트 없을 때 오류 중단 대신 신규 시트 자동 생성으로 변경
- dae_il 결과/조서 파일 업데이트
- graphy 조서 파일명 변경(당기_graphy_25년 → 당기_graphy_조서_25년) 및 results 추가
- graphy task_list_graphy.xlsx 추가

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dae_il/results/이자비용적정성.xlsx
+++ b/dae_il/results/이자비용적정성.xlsx
@@ -1,14 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_73A65DF2C20CBCBC4A89BBD1684E3AEBA63C32F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="하나 장기운전자금4(29320)" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="하나_장기운전자금-34142 _ 하나 장기운전자금-341" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="이자비용" state="visible" r:id="rId6"/>
+    <sheet name="하나 장기운전자금4(29320)" sheetId="1" r:id="rId1"/>
+    <sheet name="하나_장기운전자금-34142 _ 하나 장기운전자금-341" sheetId="2" r:id="rId2"/>
+    <sheet name="이자비용" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1137,14 +1154,21 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1172,7 +1196,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1508,11 +1532,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1538,7 +1562,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -1550,17 +1574,18 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1586,7 +1611,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>10</v>
       </c>
@@ -1597,12 +1622,12 @@
         <v>2000000000</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="1">
-        <v>46112.00060185185</v>
+        <v>46112.000601851847</v>
       </c>
       <c r="D3" t="s">
         <v>11</v>
@@ -1618,17 +1643,18 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H314"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1654,12 +1680,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>14</v>
       </c>
       <c r="C2" s="1">
-        <v>46024.00060185185</v>
+        <v>46024.000601851847</v>
       </c>
       <c r="D2" t="s">
         <v>15</v>
@@ -1674,12 +1700,12 @@
         <v>1566315</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="1">
-        <v>46035.00060185185</v>
+        <v>46035.000601851847</v>
       </c>
       <c r="D3" t="s">
         <v>18</v>
@@ -1694,12 +1720,12 @@
         <v>4119123</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="1">
-        <v>46037.00060185185</v>
+        <v>46037.000601851847</v>
       </c>
       <c r="D4" t="s">
         <v>21</v>
@@ -1714,12 +1740,12 @@
         <v>3971382</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="1">
-        <v>46037.00060185185</v>
+        <v>46037.000601851847</v>
       </c>
       <c r="D5" t="s">
         <v>24</v>
@@ -1734,12 +1760,12 @@
         <v>17978501</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="1">
-        <v>46037.00060185185</v>
+        <v>46037.000601851847</v>
       </c>
       <c r="D6" t="s">
         <v>27</v>
@@ -1754,12 +1780,12 @@
         <v>3826367</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="1">
-        <v>46037.00060185185</v>
+        <v>46037.000601851847</v>
       </c>
       <c r="D7" t="s">
         <v>30</v>
@@ -1774,12 +1800,12 @@
         <v>777319</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="1">
-        <v>46038.00060185185</v>
+        <v>46038.000601851847</v>
       </c>
       <c r="D8" t="s">
         <v>33</v>
@@ -1794,12 +1820,12 @@
         <v>7516016</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>14</v>
       </c>
       <c r="C9" s="1">
-        <v>46039.00060185185</v>
+        <v>46039.000601851847</v>
       </c>
       <c r="D9" t="s">
         <v>36</v>
@@ -1814,12 +1840,12 @@
         <v>14283556</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="1">
-        <v>46042.00060185185</v>
+        <v>46042.000601851847</v>
       </c>
       <c r="D10" t="s">
         <v>39</v>
@@ -1834,12 +1860,12 @@
         <v>3600362</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>14</v>
       </c>
       <c r="C11" s="1">
-        <v>46043.00060185185</v>
+        <v>46043.000601851847</v>
       </c>
       <c r="D11" t="s">
         <v>42</v>
@@ -1854,12 +1880,12 @@
         <v>11485183</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>14</v>
       </c>
       <c r="C12" s="1">
-        <v>46053.00060185185</v>
+        <v>46053.000601851847</v>
       </c>
       <c r="D12" t="s">
         <v>45</v>
@@ -1874,12 +1900,12 @@
         <v>19798673</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>14</v>
       </c>
       <c r="C13" s="1">
-        <v>46053.00060185185</v>
+        <v>46053.000601851847</v>
       </c>
       <c r="D13" t="s">
         <v>48</v>
@@ -1894,12 +1920,12 @@
         <v>1168482</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="1">
-        <v>46053.00060185185</v>
+        <v>46053.000601851847</v>
       </c>
       <c r="D14" t="s">
         <v>51</v>
@@ -1914,12 +1940,12 @@
         <v>3183867</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>14</v>
       </c>
       <c r="C15" s="1">
-        <v>46053.00060185185</v>
+        <v>46053.000601851847</v>
       </c>
       <c r="D15" t="s">
         <v>54</v>
@@ -1934,12 +1960,12 @@
         <v>10482881</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>14</v>
       </c>
       <c r="C16" s="1">
-        <v>46053.00060185185</v>
+        <v>46053.000601851847</v>
       </c>
       <c r="D16" t="s">
         <v>57</v>
@@ -1954,12 +1980,12 @@
         <v>1420403</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>14</v>
       </c>
       <c r="C17" s="1">
-        <v>46053.00060185185</v>
+        <v>46053.000601851847</v>
       </c>
       <c r="D17" t="s">
         <v>60</v>
@@ -1974,12 +2000,12 @@
         <v>7645210</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>14</v>
       </c>
       <c r="C18" s="1">
-        <v>46053.00060185185</v>
+        <v>46053.000601851847</v>
       </c>
       <c r="D18" t="s">
         <v>61</v>
@@ -1994,12 +2020,12 @@
         <v>3598209</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>14</v>
       </c>
       <c r="C19" s="1">
-        <v>46056.00060185185</v>
+        <v>46056.000601851847</v>
       </c>
       <c r="D19" t="s">
         <v>64</v>
@@ -2014,12 +2040,12 @@
         <v>1570468</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>14</v>
       </c>
       <c r="C20" s="1">
-        <v>46065.00060185185</v>
+        <v>46065.000601851847</v>
       </c>
       <c r="D20" t="s">
         <v>65</v>
@@ -2034,12 +2060,12 @@
         <v>4126397</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>14</v>
       </c>
       <c r="C21" s="1">
-        <v>46070.00060185185</v>
+        <v>46070.000601851847</v>
       </c>
       <c r="D21" t="s">
         <v>66</v>
@@ -2054,12 +2080,12 @@
         <v>3977342</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>14</v>
       </c>
       <c r="C22" s="1">
-        <v>46070.00060185185</v>
+        <v>46070.000601851847</v>
       </c>
       <c r="D22" t="s">
         <v>67</v>
@@ -2074,12 +2100,12 @@
         <v>18005479</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>14</v>
       </c>
       <c r="C23" s="1">
-        <v>46070.00060185185</v>
+        <v>46070.000601851847</v>
       </c>
       <c r="D23" t="s">
         <v>68</v>
@@ -2094,12 +2120,12 @@
         <v>3832109</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>14</v>
       </c>
       <c r="C24" s="1">
-        <v>46070.00060185185</v>
+        <v>46070.000601851847</v>
       </c>
       <c r="D24" t="s">
         <v>69</v>
@@ -2114,12 +2140,12 @@
         <v>766421</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>14</v>
       </c>
       <c r="C25" s="1">
-        <v>46070.00060185185</v>
+        <v>46070.000601851847</v>
       </c>
       <c r="D25" t="s">
         <v>70</v>
@@ -2134,12 +2160,12 @@
         <v>6811506</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>14</v>
       </c>
       <c r="C26" s="1">
-        <v>46070.00060185185</v>
+        <v>46070.000601851847</v>
       </c>
       <c r="D26" t="s">
         <v>71</v>
@@ -2154,12 +2180,12 @@
         <v>14302465</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>14</v>
       </c>
       <c r="C27" s="1">
-        <v>46072.00060185185</v>
+        <v>46072.000601851847</v>
       </c>
       <c r="D27" t="s">
         <v>72</v>
@@ -2174,12 +2200,12 @@
         <v>3604493</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>14</v>
       </c>
       <c r="C28" s="1">
-        <v>46074.00060185185</v>
+        <v>46074.000601851847</v>
       </c>
       <c r="D28" t="s">
         <v>73</v>
@@ -2194,12 +2220,12 @@
         <v>11496328</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>14</v>
       </c>
       <c r="C29" s="1">
-        <v>46080.00060185185</v>
+        <v>46080.000601851847</v>
       </c>
       <c r="D29" t="s">
         <v>74</v>
@@ -2214,12 +2240,12 @@
         <v>1168997</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>14</v>
       </c>
       <c r="C30" s="1">
-        <v>46080.00060185185</v>
+        <v>46080.000601851847</v>
       </c>
       <c r="D30" t="s">
         <v>75</v>
@@ -2234,12 +2260,12 @@
         <v>3185271</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>14</v>
       </c>
       <c r="C31" s="1">
-        <v>46080.00060185185</v>
+        <v>46080.000601851847</v>
       </c>
       <c r="D31" t="s">
         <v>76</v>
@@ -2254,12 +2280,12 @@
         <v>19807403</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>14</v>
       </c>
       <c r="C32" s="1">
-        <v>46081.00060185185</v>
+        <v>46081.000601851847</v>
       </c>
       <c r="D32" t="s">
         <v>77</v>
@@ -2274,12 +2300,12 @@
         <v>9658750</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>14</v>
       </c>
       <c r="C33" s="1">
-        <v>46081.00060185185</v>
+        <v>46081.000601851847</v>
       </c>
       <c r="D33" t="s">
         <v>78</v>
@@ -2294,12 +2320,12 @@
         <v>1312259</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>14</v>
       </c>
       <c r="C34" s="1">
-        <v>46081.00060185185</v>
+        <v>46081.000601851847</v>
       </c>
       <c r="D34" t="s">
         <v>79</v>
@@ -2314,12 +2340,12 @@
         <v>7400547</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>14</v>
       </c>
       <c r="C35" s="1">
-        <v>46081.00060185185</v>
+        <v>46081.000601851847</v>
       </c>
       <c r="D35" t="s">
         <v>80</v>
@@ -2334,12 +2360,12 @@
         <v>3476712</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>14</v>
       </c>
       <c r="C36" s="1">
-        <v>46085.00060185185</v>
+        <v>46085.000601851847</v>
       </c>
       <c r="D36" t="s">
         <v>81</v>
@@ -2354,12 +2380,12 @@
         <v>1418487</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>14</v>
       </c>
       <c r="C37" s="1">
-        <v>46093.00060185185</v>
+        <v>46093.000601851847</v>
       </c>
       <c r="D37" t="s">
         <v>82</v>
@@ -2374,12 +2400,12 @@
         <v>3727068</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>14</v>
       </c>
       <c r="C38" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D38" t="s">
         <v>83</v>
@@ -2394,12 +2420,12 @@
         <v>3849041</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>14</v>
       </c>
       <c r="C39" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D39" t="s">
         <v>84</v>
@@ -2414,12 +2440,12 @@
         <v>16263013</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>14</v>
       </c>
       <c r="C40" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D40" t="s">
         <v>85</v>
@@ -2434,12 +2460,12 @@
         <v>3461260</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>14</v>
       </c>
       <c r="C41" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D41" t="s">
         <v>86</v>
@@ -2454,12 +2480,12 @@
         <v>10109015</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>14</v>
       </c>
       <c r="C42" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D42" t="s">
         <v>89</v>
@@ -2474,12 +2500,12 @@
         <v>9763942</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>14</v>
       </c>
       <c r="C43" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D43" t="s">
         <v>92</v>
@@ -2494,12 +2520,12 @@
         <v>692252</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>14</v>
       </c>
       <c r="C44" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D44" t="s">
         <v>93</v>
@@ -2514,12 +2540,12 @@
         <v>7444506</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>14</v>
       </c>
       <c r="C45" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D45" t="s">
         <v>96</v>
@@ -2534,12 +2560,12 @@
         <v>3727872</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>14</v>
       </c>
       <c r="C46" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D46" t="s">
         <v>97</v>
@@ -2554,12 +2580,12 @@
         <v>2572918</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>14</v>
       </c>
       <c r="C47" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D47" t="s">
         <v>98</v>
@@ -2574,12 +2600,12 @@
         <v>6747502</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>14</v>
       </c>
       <c r="C48" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D48" t="s">
         <v>99</v>
@@ -2594,12 +2620,12 @@
         <v>1422570</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>14</v>
       </c>
       <c r="C49" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D49" t="s">
         <v>100</v>
@@ -2614,12 +2640,12 @@
         <v>4291893</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>14</v>
       </c>
       <c r="C50" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D50" t="s">
         <v>103</v>
@@ -2634,12 +2660,12 @@
         <v>2861262</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>14</v>
       </c>
       <c r="C51" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D51" t="s">
         <v>100</v>
@@ -2654,12 +2680,12 @@
         <v>4291893</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>14</v>
       </c>
       <c r="C52" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D52" t="s">
         <v>104</v>
@@ -2674,12 +2700,12 @@
         <v>811109</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>14</v>
       </c>
       <c r="C53" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D53" t="s">
         <v>105</v>
@@ -2694,12 +2720,12 @@
         <v>6152328</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>14</v>
       </c>
       <c r="C54" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D54" t="s">
         <v>106</v>
@@ -2714,12 +2740,12 @@
         <v>25492021</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>14</v>
       </c>
       <c r="C55" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D55" t="s">
         <v>109</v>
@@ -2734,12 +2760,12 @@
         <v>11471409</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>14</v>
       </c>
       <c r="C56" s="1">
-        <v>46098.00060185185</v>
+        <v>46098.000601851847</v>
       </c>
       <c r="D56" t="s">
         <v>112</v>
@@ -2754,12 +2780,12 @@
         <v>12918356</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>14</v>
       </c>
       <c r="C57" s="1">
-        <v>46100.00060185185</v>
+        <v>46100.000601851847</v>
       </c>
       <c r="D57" t="s">
         <v>113</v>
@@ -2774,12 +2800,12 @@
         <v>3255671</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>14</v>
       </c>
       <c r="C58" s="1">
-        <v>46102.00060185185</v>
+        <v>46102.000601851847</v>
       </c>
       <c r="D58" t="s">
         <v>114</v>
@@ -2794,12 +2820,12 @@
         <v>10383780</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>14</v>
       </c>
       <c r="C59" s="1">
-        <v>46108.00060185185</v>
+        <v>46108.000601851847</v>
       </c>
       <c r="D59" t="s">
         <v>115</v>
@@ -2814,12 +2840,12 @@
         <v>17890557</v>
       </c>
     </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>14</v>
       </c>
       <c r="C60" s="1">
-        <v>46108.00060185185</v>
+        <v>46108.000601851847</v>
       </c>
       <c r="D60" t="s">
         <v>116</v>
@@ -2834,12 +2860,12 @@
         <v>1055868</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>14</v>
       </c>
       <c r="C61" s="1">
-        <v>46108.00060185185</v>
+        <v>46108.000601851847</v>
       </c>
       <c r="D61" t="s">
         <v>117</v>
@@ -2854,12 +2880,12 @@
         <v>2877019</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>14</v>
       </c>
       <c r="C62" s="1">
-        <v>46109.00060185185</v>
+        <v>46109.000601851847</v>
       </c>
       <c r="D62" t="s">
         <v>118</v>
@@ -2874,12 +2900,12 @@
         <v>8724032</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>14</v>
       </c>
       <c r="C63" s="1">
-        <v>46109.00060185185</v>
+        <v>46109.000601851847</v>
       </c>
       <c r="D63" t="s">
         <v>119</v>
@@ -2894,12 +2920,12 @@
         <v>1006849</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>14</v>
       </c>
       <c r="C64" s="1">
-        <v>46109.00060185185</v>
+        <v>46109.000601851847</v>
       </c>
       <c r="D64" t="s">
         <v>120</v>
@@ -2914,12 +2940,12 @@
         <v>3244931</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>14</v>
       </c>
       <c r="C65" s="1">
-        <v>46112.00060185185</v>
+        <v>46112.000601851847</v>
       </c>
       <c r="D65" t="s">
         <v>121</v>
@@ -2934,12 +2960,12 @@
         <v>6877040</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>14</v>
       </c>
       <c r="C66" s="1">
-        <v>46112.00060185185</v>
+        <v>46112.000601851847</v>
       </c>
       <c r="D66" t="s">
         <v>122</v>
@@ -2954,12 +2980,12 @@
         <v>2637192</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>14</v>
       </c>
       <c r="C67" s="1">
-        <v>46112.00060185185</v>
+        <v>46112.000601851847</v>
       </c>
       <c r="D67" t="s">
         <v>125</v>
@@ -2974,12 +3000,12 @@
         <v>2569571</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>14</v>
       </c>
       <c r="C68" s="1">
-        <v>46112.00060185185</v>
+        <v>46112.000601851847</v>
       </c>
       <c r="D68" t="s">
         <v>126</v>
@@ -2994,12 +3020,12 @@
         <v>954639</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>14</v>
       </c>
       <c r="C69" s="1">
-        <v>46112.00060185185</v>
+        <v>46112.000601851847</v>
       </c>
       <c r="D69" t="s">
         <v>127</v>
@@ -3014,12 +3040,12 @@
         <v>1014304</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>14</v>
       </c>
       <c r="C70" s="1">
-        <v>46112.00060185185</v>
+        <v>46112.000601851847</v>
       </c>
       <c r="D70" t="s">
         <v>128</v>
@@ -3034,12 +3060,12 @@
         <v>715979</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>14</v>
       </c>
       <c r="C71" s="1">
-        <v>46112.00060185185</v>
+        <v>46112.000601851847</v>
       </c>
       <c r="D71" t="s">
         <v>129</v>
@@ -3054,12 +3080,12 @@
         <v>636426</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>14</v>
       </c>
       <c r="C72" s="1">
-        <v>46112.00060185185</v>
+        <v>46112.000601851847</v>
       </c>
       <c r="D72" t="s">
         <v>130</v>
@@ -3074,12 +3100,12 @@
         <v>122977</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>14</v>
       </c>
       <c r="C73" s="1">
-        <v>46114.00060185185</v>
+        <v>46114.000601851847</v>
       </c>
       <c r="D73" t="s">
         <v>131</v>
@@ -3094,12 +3120,12 @@
         <v>1391303</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>14</v>
       </c>
       <c r="C74" s="1">
-        <v>46115.00060185185</v>
+        <v>46115.000601851847</v>
       </c>
       <c r="D74" t="s">
         <v>121</v>
@@ -3114,12 +3140,12 @@
         <v>649644</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>14</v>
       </c>
       <c r="C75" s="1">
-        <v>46126.00060185185</v>
+        <v>46126.000601851847</v>
       </c>
       <c r="D75" t="s">
         <v>132</v>
@@ -3134,12 +3160,12 @@
         <v>4126397</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>14</v>
       </c>
       <c r="C76" s="1">
-        <v>46127.00060185185</v>
+        <v>46127.000601851847</v>
       </c>
       <c r="D76" t="s">
         <v>133</v>
@@ -3154,12 +3180,12 @@
         <v>17886575</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
         <v>14</v>
       </c>
       <c r="C77" s="1">
-        <v>46127.00060185185</v>
+        <v>46127.000601851847</v>
       </c>
       <c r="D77" t="s">
         <v>134</v>
@@ -3174,12 +3200,12 @@
         <v>3424438</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
         <v>14</v>
       </c>
       <c r="C78" s="1">
-        <v>46127.00060185185</v>
+        <v>46127.000601851847</v>
       </c>
       <c r="D78" t="s">
         <v>135</v>
@@ -3194,12 +3220,12 @@
         <v>364536</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
         <v>14</v>
       </c>
       <c r="C79" s="1">
-        <v>46128.00060185185</v>
+        <v>46128.000601851847</v>
       </c>
       <c r="D79" t="s">
         <v>136</v>
@@ -3214,12 +3240,12 @@
         <v>6811506</v>
       </c>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
         <v>14</v>
       </c>
       <c r="C80" s="1">
-        <v>46129.00060185185</v>
+        <v>46129.000601851847</v>
       </c>
       <c r="D80" t="s">
         <v>137</v>
@@ -3234,12 +3260,12 @@
         <v>14302465</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
         <v>14</v>
       </c>
       <c r="C81" s="1">
-        <v>46129.00060185185</v>
+        <v>46129.000601851847</v>
       </c>
       <c r="D81" t="s">
         <v>138</v>
@@ -3254,12 +3280,12 @@
         <v>3873726</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
         <v>14</v>
       </c>
       <c r="C82" s="1">
-        <v>46133.00060185185</v>
+        <v>46133.000601851847</v>
       </c>
       <c r="D82" t="s">
         <v>139</v>
@@ -3274,12 +3300,12 @@
         <v>3604493</v>
       </c>
     </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
         <v>14</v>
       </c>
       <c r="C83" s="1">
-        <v>46133.00060185185</v>
+        <v>46133.000601851847</v>
       </c>
       <c r="D83" t="s">
         <v>140</v>
@@ -3294,12 +3320,12 @@
         <v>11496328</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
         <v>14</v>
       </c>
       <c r="C84" s="1">
-        <v>46140.00060185185</v>
+        <v>46140.000601851847</v>
       </c>
       <c r="D84" t="s">
         <v>141</v>
@@ -3314,12 +3340,12 @@
         <v>19807403</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
         <v>14</v>
       </c>
       <c r="C85" s="1">
-        <v>46140.00060185185</v>
+        <v>46140.000601851847</v>
       </c>
       <c r="D85" t="s">
         <v>142</v>
@@ -3334,12 +3360,12 @@
         <v>1028860</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>14</v>
       </c>
       <c r="C86" s="1">
-        <v>46140.00060185185</v>
+        <v>46140.000601851847</v>
       </c>
       <c r="D86" t="s">
         <v>143</v>
@@ -3354,12 +3380,12 @@
         <v>2811572</v>
       </c>
     </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
         <v>14</v>
       </c>
       <c r="C87" s="1">
-        <v>46140.00060185185</v>
+        <v>46140.000601851847</v>
       </c>
       <c r="D87" t="s">
         <v>144</v>
@@ -3374,12 +3400,12 @@
         <v>9658750</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
         <v>14</v>
       </c>
       <c r="C88" s="1">
-        <v>46140.00060185185</v>
+        <v>46140.000601851847</v>
       </c>
       <c r="D88" t="s">
         <v>145</v>
@@ -3394,12 +3420,12 @@
         <v>1114726</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
         <v>14</v>
       </c>
       <c r="C89" s="1">
-        <v>46140.00060185185</v>
+        <v>46140.000601851847</v>
       </c>
       <c r="D89" t="s">
         <v>146</v>
@@ -3414,12 +3440,12 @@
         <v>3592602</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
         <v>14</v>
       </c>
       <c r="C90" s="1">
-        <v>46142.00060185185</v>
+        <v>46142.000601851847</v>
       </c>
       <c r="D90" t="s">
         <v>147</v>
@@ -3434,12 +3460,12 @@
         <v>7351232</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
         <v>14</v>
       </c>
       <c r="C91" s="1">
-        <v>46144.00060185185</v>
+        <v>46144.000601851847</v>
       </c>
       <c r="D91" t="s">
         <v>148</v>
@@ -3454,12 +3480,12 @@
         <v>1334465</v>
       </c>
     </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
         <v>14</v>
       </c>
       <c r="C92" s="1">
-        <v>46149.00060185185</v>
+        <v>46149.000601851847</v>
       </c>
       <c r="D92" t="s">
         <v>149</v>
@@ -3474,12 +3500,12 @@
         <v>61047</v>
       </c>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>14</v>
       </c>
       <c r="C93" s="1">
-        <v>46154.00060185185</v>
+        <v>46154.000601851847</v>
       </c>
       <c r="D93" t="s">
         <v>152</v>
@@ -3494,12 +3520,12 @@
         <v>3993287</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
         <v>14</v>
       </c>
       <c r="C94" s="1">
-        <v>46157.00060185185</v>
+        <v>46157.000601851847</v>
       </c>
       <c r="D94" t="s">
         <v>154</v>
@@ -3514,12 +3540,12 @@
         <v>17309589</v>
       </c>
     </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
         <v>14</v>
       </c>
       <c r="C95" s="1">
-        <v>46157.00060185185</v>
+        <v>46157.000601851847</v>
       </c>
       <c r="D95" t="s">
         <v>155</v>
@@ -3534,12 +3560,12 @@
         <v>3313972</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
         <v>14</v>
       </c>
       <c r="C96" s="1">
-        <v>46157.00060185185</v>
+        <v>46157.000601851847</v>
       </c>
       <c r="D96" t="s">
         <v>156</v>
@@ -3554,12 +3580,12 @@
         <v>331397</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>14</v>
       </c>
       <c r="C97" s="1">
-        <v>46158.00060185185</v>
+        <v>46158.000601851847</v>
       </c>
       <c r="D97" t="s">
         <v>157</v>
@@ -3574,12 +3600,12 @@
         <v>6147945</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>14</v>
       </c>
       <c r="C98" s="1">
-        <v>46161.00060185185</v>
+        <v>46161.000601851847</v>
       </c>
       <c r="D98" t="s">
         <v>158</v>
@@ -3594,12 +3620,12 @@
         <v>3748767</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
         <v>14</v>
       </c>
       <c r="C99" s="1">
-        <v>46161.00060185185</v>
+        <v>46161.000601851847</v>
       </c>
       <c r="D99" t="s">
         <v>159</v>
@@ -3614,12 +3640,12 @@
         <v>3488219</v>
       </c>
     </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>14</v>
       </c>
       <c r="C100" s="1">
-        <v>46161.00060185185</v>
+        <v>46161.000601851847</v>
       </c>
       <c r="D100" t="s">
         <v>137</v>
@@ -3634,12 +3660,12 @@
         <v>13841095</v>
       </c>
     </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>14</v>
       </c>
       <c r="C101" s="1">
-        <v>46164.00060185185</v>
+        <v>46164.000601851847</v>
       </c>
       <c r="D101" t="s">
         <v>160</v>
@@ -3654,12 +3680,12 @@
         <v>10444931</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>14</v>
       </c>
       <c r="C102" s="1">
-        <v>46169.00060185185</v>
+        <v>46169.000601851847</v>
       </c>
       <c r="D102" t="s">
         <v>161</v>
@@ -3674,12 +3700,12 @@
         <v>995671</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>14</v>
       </c>
       <c r="C103" s="1">
-        <v>46169.00060185185</v>
+        <v>46169.000601851847</v>
       </c>
       <c r="D103" t="s">
         <v>162</v>
@@ -3694,12 +3720,12 @@
         <v>2720876</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
         <v>14</v>
       </c>
       <c r="C104" s="1">
-        <v>46169.00060185185</v>
+        <v>46169.000601851847</v>
       </c>
       <c r="D104" t="s">
         <v>163</v>
@@ -3714,12 +3740,12 @@
         <v>19168454</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>14</v>
       </c>
       <c r="C105" s="1">
-        <v>46170.00060185185</v>
+        <v>46170.000601851847</v>
       </c>
       <c r="D105" t="s">
         <v>164</v>
@@ -3734,12 +3760,12 @@
         <v>8659232</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>14</v>
       </c>
       <c r="C106" s="1">
-        <v>46170.00060185185</v>
+        <v>46170.000601851847</v>
       </c>
       <c r="D106" t="s">
         <v>165</v>
@@ -3754,12 +3780,12 @@
         <v>1078767</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>14</v>
       </c>
       <c r="C107" s="1">
-        <v>46170.00060185185</v>
+        <v>46170.000601851847</v>
       </c>
       <c r="D107" t="s">
         <v>166</v>
@@ -3774,12 +3800,12 @@
         <v>3476712</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>14</v>
       </c>
       <c r="C108" s="1">
-        <v>46175.00060185185</v>
+        <v>46175.000601851847</v>
       </c>
       <c r="D108" t="s">
         <v>167</v>
@@ -3794,12 +3820,12 @@
         <v>1378947</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>14</v>
       </c>
       <c r="C109" s="1">
-        <v>46175.00060185185</v>
+        <v>46175.000601851847</v>
       </c>
       <c r="D109" t="s">
         <v>168</v>
@@ -3814,12 +3840,12 @@
         <v>7596273</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>14</v>
       </c>
       <c r="C110" s="1">
-        <v>46182.00060185185</v>
+        <v>46182.000601851847</v>
       </c>
       <c r="D110" t="s">
         <v>169</v>
@@ -3834,12 +3860,12 @@
         <v>116788</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>14</v>
       </c>
       <c r="C111" s="1">
-        <v>46185.00060185185</v>
+        <v>46185.000601851847</v>
       </c>
       <c r="D111" t="s">
         <v>170</v>
@@ -3854,12 +3880,12 @@
         <v>4126397</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
         <v>14</v>
       </c>
       <c r="C112" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D112" t="s">
         <v>171</v>
@@ -3874,12 +3900,12 @@
         <v>17886575</v>
       </c>
     </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>14</v>
       </c>
       <c r="C113" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D113" t="s">
         <v>172</v>
@@ -3894,12 +3920,12 @@
         <v>3424438</v>
       </c>
     </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>14</v>
       </c>
       <c r="C114" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D114" t="s">
         <v>173</v>
@@ -3914,12 +3940,12 @@
         <v>9539176</v>
       </c>
     </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>14</v>
       </c>
       <c r="C115" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D115" t="s">
         <v>174</v>
@@ -3934,12 +3960,12 @@
         <v>9191538</v>
       </c>
     </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>14</v>
       </c>
       <c r="C116" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D116" t="s">
         <v>175</v>
@@ -3954,12 +3980,12 @@
         <v>352722</v>
       </c>
     </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>14</v>
       </c>
       <c r="C117" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D117" t="s">
         <v>176</v>
@@ -3974,12 +4000,12 @@
         <v>7613869</v>
       </c>
     </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>14</v>
       </c>
       <c r="C118" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D118" t="s">
         <v>177</v>
@@ -3994,12 +4020,12 @@
         <v>3812681</v>
       </c>
     </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>14</v>
       </c>
       <c r="C119" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D119" t="s">
         <v>178</v>
@@ -4014,12 +4040,12 @@
         <v>2631452</v>
       </c>
     </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>14</v>
       </c>
       <c r="C120" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D120" t="s">
         <v>179</v>
@@ -4034,12 +4060,12 @@
         <v>6901008</v>
       </c>
     </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>14</v>
       </c>
       <c r="C121" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D121" t="s">
         <v>180</v>
@@ -4054,12 +4080,12 @@
         <v>1657008</v>
       </c>
     </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>14</v>
       </c>
       <c r="C122" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D122" t="s">
         <v>181</v>
@@ -4074,12 +4100,12 @@
         <v>4389534</v>
       </c>
     </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>14</v>
       </c>
       <c r="C123" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D123" t="s">
         <v>182</v>
@@ -4094,12 +4120,12 @@
         <v>2926356</v>
       </c>
     </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>14</v>
       </c>
       <c r="C124" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D124" t="s">
         <v>181</v>
@@ -4114,12 +4140,12 @@
         <v>4389534</v>
       </c>
     </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>14</v>
       </c>
       <c r="C125" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D125" t="s">
         <v>183</v>
@@ -4134,12 +4160,12 @@
         <v>1463178</v>
       </c>
     </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>14</v>
       </c>
       <c r="C126" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D126" t="s">
         <v>184</v>
@@ -4154,12 +4180,12 @@
         <v>1989847</v>
       </c>
     </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>14</v>
       </c>
       <c r="C127" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D127" t="s">
         <v>187</v>
@@ -4174,12 +4200,12 @@
         <v>184924</v>
       </c>
     </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>14</v>
       </c>
       <c r="C128" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D128" t="s">
         <v>188</v>
@@ -4194,12 +4220,12 @@
         <v>6352876</v>
       </c>
     </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>14</v>
       </c>
       <c r="C129" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D129" t="s">
         <v>189</v>
@@ -4214,12 +4240,12 @@
         <v>24530957</v>
       </c>
     </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
         <v>14</v>
       </c>
       <c r="C130" s="1">
-        <v>46189.00060185185</v>
+        <v>46189.000601851847</v>
       </c>
       <c r="D130" t="s">
         <v>190</v>
@@ -4234,12 +4260,12 @@
         <v>11038930</v>
       </c>
     </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>14</v>
       </c>
       <c r="C131" s="1">
-        <v>46190.00060185185</v>
+        <v>46190.000601851847</v>
       </c>
       <c r="D131" t="s">
         <v>191</v>
@@ -4254,12 +4280,12 @@
         <v>14302465</v>
       </c>
     </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>14</v>
       </c>
       <c r="C132" s="1">
-        <v>46190.00060185185</v>
+        <v>46190.000601851847</v>
       </c>
       <c r="D132" t="s">
         <v>192</v>
@@ -4274,12 +4300,12 @@
         <v>3873724</v>
       </c>
     </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
         <v>14</v>
       </c>
       <c r="C133" s="1">
-        <v>46192.00060185185</v>
+        <v>46192.000601851847</v>
       </c>
       <c r="D133" t="s">
         <v>193</v>
@@ -4294,12 +4320,12 @@
         <v>3604493</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>14</v>
       </c>
       <c r="C134" s="1">
-        <v>46196.00060185185</v>
+        <v>46196.000601851847</v>
       </c>
       <c r="D134" t="s">
         <v>194</v>
@@ -4314,12 +4340,12 @@
         <v>10793095</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>14</v>
       </c>
       <c r="C135" s="1">
-        <v>46200.00060185185</v>
+        <v>46200.000601851847</v>
       </c>
       <c r="D135" t="s">
         <v>195</v>
@@ -4334,12 +4360,12 @@
         <v>19807403</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>14</v>
       </c>
       <c r="C136" s="1">
-        <v>46200.00060185185</v>
+        <v>46200.000601851847</v>
       </c>
       <c r="D136" t="s">
         <v>196</v>
@@ -4354,12 +4380,12 @@
         <v>1028860</v>
       </c>
     </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>14</v>
       </c>
       <c r="C137" s="1">
-        <v>46200.00060185185</v>
+        <v>46200.000601851847</v>
       </c>
       <c r="D137" t="s">
         <v>197</v>
@@ -4374,12 +4400,12 @@
         <v>2811572</v>
       </c>
     </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>14</v>
       </c>
       <c r="C138" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D138" t="s">
         <v>198</v>
@@ -4394,12 +4420,12 @@
         <v>8947873</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>14</v>
       </c>
       <c r="C139" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D139" t="s">
         <v>199</v>
@@ -4414,12 +4440,12 @@
         <v>1114726</v>
       </c>
     </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>14</v>
       </c>
       <c r="C140" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D140" t="s">
         <v>200</v>
@@ -4434,12 +4460,12 @@
         <v>7351232</v>
       </c>
     </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>14</v>
       </c>
       <c r="C141" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D141" t="s">
         <v>201</v>
@@ -4454,12 +4480,12 @@
         <v>2612219</v>
       </c>
     </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>14</v>
       </c>
       <c r="C142" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D142" t="s">
         <v>202</v>
@@ -4474,12 +4500,12 @@
         <v>2545239</v>
       </c>
     </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
         <v>14</v>
       </c>
       <c r="C143" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D143" t="s">
         <v>203</v>
@@ -4494,12 +4520,12 @@
         <v>945599</v>
       </c>
     </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>14</v>
       </c>
       <c r="C144" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D144" t="s">
         <v>204</v>
@@ -4514,12 +4540,12 @@
         <v>1004699</v>
       </c>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>14</v>
       </c>
       <c r="C145" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D145" t="s">
         <v>205</v>
@@ -4534,12 +4560,12 @@
         <v>709199</v>
       </c>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>14</v>
       </c>
       <c r="C146" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D146" t="s">
         <v>206</v>
@@ -4554,12 +4580,12 @@
         <v>630399</v>
       </c>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>14</v>
       </c>
       <c r="C147" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D147" t="s">
         <v>207</v>
@@ -4574,12 +4600,12 @@
         <v>267919</v>
       </c>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>14</v>
       </c>
       <c r="C148" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D148" t="s">
         <v>208</v>
@@ -4594,12 +4620,12 @@
         <v>4462352</v>
       </c>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>14</v>
       </c>
       <c r="C149" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D149" t="s">
         <v>211</v>
@@ -4614,12 +4640,12 @@
         <v>2651543</v>
       </c>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>14</v>
       </c>
       <c r="C150" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D150" t="s">
         <v>212</v>
@@ -4634,12 +4660,12 @@
         <v>696065</v>
       </c>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>14</v>
       </c>
       <c r="C151" s="1">
-        <v>46203.00060185185</v>
+        <v>46203.000601851847</v>
       </c>
       <c r="D151" t="s">
         <v>213</v>
@@ -4654,12 +4680,12 @@
         <v>3824383</v>
       </c>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>14</v>
       </c>
       <c r="C152" s="1">
-        <v>46205.00060185185</v>
+        <v>46205.000601851847</v>
       </c>
       <c r="D152" t="s">
         <v>214</v>
@@ -4674,12 +4700,12 @@
         <v>1207890</v>
       </c>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>14</v>
       </c>
       <c r="C153" s="1">
-        <v>46210.00060185185</v>
+        <v>46210.000601851847</v>
       </c>
       <c r="D153" t="s">
         <v>215</v>
@@ -4694,12 +4720,12 @@
         <v>1257120</v>
       </c>
     </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>14</v>
       </c>
       <c r="C154" s="1">
-        <v>46217.00060185185</v>
+        <v>46217.000601851847</v>
       </c>
       <c r="D154" t="s">
         <v>216</v>
@@ -4714,12 +4740,12 @@
         <v>3993287</v>
       </c>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>14</v>
       </c>
       <c r="C155" s="1">
-        <v>46218.00060185185</v>
+        <v>46218.000601851847</v>
       </c>
       <c r="D155" t="s">
         <v>217</v>
@@ -4734,12 +4760,12 @@
         <v>16158904</v>
       </c>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>14</v>
       </c>
       <c r="C156" s="1">
-        <v>46218.00060185185</v>
+        <v>46218.000601851847</v>
       </c>
       <c r="D156" t="s">
         <v>218</v>
@@ -4754,12 +4780,12 @@
         <v>3083835</v>
       </c>
     </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>14</v>
       </c>
       <c r="C157" s="1">
-        <v>46219.00060185185</v>
+        <v>46219.000601851847</v>
       </c>
       <c r="D157" t="s">
         <v>219</v>
@@ -4774,12 +4800,12 @@
         <v>6147945</v>
       </c>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>14</v>
       </c>
       <c r="C158" s="1">
-        <v>46220.00060185185</v>
+        <v>46220.000601851847</v>
       </c>
       <c r="D158" t="s">
         <v>220</v>
@@ -4794,12 +4820,12 @@
         <v>3748767</v>
       </c>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>14</v>
       </c>
       <c r="C159" s="1">
-        <v>46220.00060185185</v>
+        <v>46220.000601851847</v>
       </c>
       <c r="D159" t="s">
         <v>221</v>
@@ -4814,12 +4840,12 @@
         <v>13841095</v>
       </c>
     </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>14</v>
       </c>
       <c r="C160" s="1">
-        <v>46224.00060185185</v>
+        <v>46224.000601851847</v>
       </c>
       <c r="D160" t="s">
         <v>222</v>
@@ -4834,12 +4860,12 @@
         <v>3488219</v>
       </c>
     </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>14</v>
       </c>
       <c r="C161" s="1">
-        <v>46224.00060185185</v>
+        <v>46224.000601851847</v>
       </c>
       <c r="D161" t="s">
         <v>223</v>
@@ -4854,12 +4880,12 @@
         <v>10444931</v>
       </c>
     </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>14</v>
       </c>
       <c r="C162" s="1">
-        <v>46231.00060185185</v>
+        <v>46231.000601851847</v>
       </c>
       <c r="D162" t="s">
         <v>224</v>
@@ -4874,12 +4900,12 @@
         <v>19168454</v>
       </c>
     </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>14</v>
       </c>
       <c r="C163" s="1">
-        <v>46231.00060185185</v>
+        <v>46231.000601851847</v>
       </c>
       <c r="D163" t="s">
         <v>225</v>
@@ -4894,12 +4920,12 @@
         <v>2536767</v>
       </c>
     </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
         <v>14</v>
       </c>
       <c r="C164" s="1">
-        <v>46231.00060185185</v>
+        <v>46231.000601851847</v>
       </c>
       <c r="D164" t="s">
         <v>226</v>
@@ -4914,12 +4940,12 @@
         <v>926630</v>
       </c>
     </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>14</v>
       </c>
       <c r="C165" s="1">
-        <v>46231.00060185185</v>
+        <v>46231.000601851847</v>
       </c>
       <c r="D165" t="s">
         <v>227</v>
@@ -4934,12 +4960,12 @@
         <v>8659232</v>
       </c>
     </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>14</v>
       </c>
       <c r="C166" s="1">
-        <v>46231.00060185185</v>
+        <v>46231.000601851847</v>
       </c>
       <c r="D166" t="s">
         <v>228</v>
@@ -4954,12 +4980,12 @@
         <v>1078767</v>
       </c>
     </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>14</v>
       </c>
       <c r="C167" s="1">
-        <v>46231.00060185185</v>
+        <v>46231.000601851847</v>
       </c>
       <c r="D167" t="s">
         <v>229</v>
@@ -4974,12 +5000,12 @@
         <v>2669589</v>
       </c>
     </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>14</v>
       </c>
       <c r="C168" s="1">
-        <v>46234.00060185185</v>
+        <v>46234.000601851847</v>
       </c>
       <c r="D168" t="s">
         <v>230</v>
@@ -4994,12 +5020,12 @@
         <v>7137643</v>
       </c>
     </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>14</v>
       </c>
       <c r="C169" s="1">
-        <v>46238.00060185185</v>
+        <v>46238.000601851847</v>
       </c>
       <c r="D169" t="s">
         <v>231</v>
@@ -5014,12 +5040,12 @@
         <v>1248153</v>
       </c>
     </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>14</v>
       </c>
       <c r="C170" s="1">
-        <v>46240.00060185185</v>
+        <v>46240.000601851847</v>
       </c>
       <c r="D170" t="s">
         <v>232</v>
@@ -5034,12 +5060,12 @@
         <v>168672</v>
       </c>
     </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>14</v>
       </c>
       <c r="C171" s="1">
-        <v>46246.00060185185</v>
+        <v>46246.000601851847</v>
       </c>
       <c r="D171" t="s">
         <v>233</v>
@@ -5054,12 +5080,12 @@
         <v>4126397</v>
       </c>
     </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
         <v>14</v>
       </c>
       <c r="C172" s="1">
-        <v>46252.00060185185</v>
+        <v>46252.000601851847</v>
       </c>
       <c r="D172" t="s">
         <v>234</v>
@@ -5074,12 +5100,12 @@
         <v>3873726</v>
       </c>
     </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
         <v>14</v>
       </c>
       <c r="C173" s="1">
-        <v>46252.00060185185</v>
+        <v>46252.000601851847</v>
       </c>
       <c r="D173" t="s">
         <v>235</v>
@@ -5094,12 +5120,12 @@
         <v>16697534</v>
       </c>
     </row>
-    <row r="174" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>14</v>
       </c>
       <c r="C174" s="1">
-        <v>46252.00060185185</v>
+        <v>46252.000601851847</v>
       </c>
       <c r="D174" t="s">
         <v>236</v>
@@ -5114,12 +5140,12 @@
         <v>3186630</v>
       </c>
     </row>
-    <row r="175" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>14</v>
       </c>
       <c r="C175" s="1">
-        <v>46252.00060185185</v>
+        <v>46252.000601851847</v>
       </c>
       <c r="D175" t="s">
         <v>237</v>
@@ -5134,12 +5160,12 @@
         <v>5996164</v>
       </c>
     </row>
-    <row r="176" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>14</v>
       </c>
       <c r="C176" s="1">
-        <v>46252.00060185185</v>
+        <v>46252.000601851847</v>
       </c>
       <c r="D176" t="s">
         <v>238</v>
@@ -5154,12 +5180,12 @@
         <v>14302465</v>
       </c>
     </row>
-    <row r="177" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A177" t="s">
         <v>14</v>
       </c>
       <c r="C177" s="1">
-        <v>46253.00060185185</v>
+        <v>46253.000601851847</v>
       </c>
       <c r="D177" t="s">
         <v>239</v>
@@ -5174,12 +5200,12 @@
         <v>3604493</v>
       </c>
     </row>
-    <row r="178" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A178" t="s">
         <v>14</v>
       </c>
       <c r="C178" s="1">
-        <v>46255.00060185185</v>
+        <v>46255.000601851847</v>
       </c>
       <c r="D178" t="s">
         <v>240</v>
@@ -5194,12 +5220,12 @@
         <v>10308986</v>
       </c>
     </row>
-    <row r="179" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A179" t="s">
         <v>14</v>
       </c>
       <c r="C179" s="1">
-        <v>46261.00060185185</v>
+        <v>46261.000601851847</v>
       </c>
       <c r="D179" t="s">
         <v>241</v>
@@ -5214,12 +5240,12 @@
         <v>19807403</v>
       </c>
     </row>
-    <row r="180" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A180" t="s">
         <v>14</v>
       </c>
       <c r="C180" s="1">
-        <v>46261.00060185185</v>
+        <v>46261.000601851847</v>
       </c>
       <c r="D180" t="s">
         <v>242</v>
@@ -5234,12 +5260,12 @@
         <v>2621326</v>
       </c>
     </row>
-    <row r="181" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A181" t="s">
         <v>14</v>
       </c>
       <c r="C181" s="1">
-        <v>46261.00060185185</v>
+        <v>46261.000601851847</v>
       </c>
       <c r="D181" t="s">
         <v>243</v>
@@ -5254,12 +5280,12 @@
         <v>957517</v>
       </c>
     </row>
-    <row r="182" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A182" t="s">
         <v>14</v>
       </c>
       <c r="C182" s="1">
-        <v>46262.00060185185</v>
+        <v>46262.000601851847</v>
       </c>
       <c r="D182" t="s">
         <v>244</v>
@@ -5274,12 +5300,12 @@
         <v>8466312</v>
       </c>
     </row>
-    <row r="183" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A183" t="s">
         <v>14</v>
       </c>
       <c r="C183" s="1">
-        <v>46262.00060185185</v>
+        <v>46262.000601851847</v>
       </c>
       <c r="D183" t="s">
         <v>245</v>
@@ -5294,12 +5320,12 @@
         <v>1114726</v>
       </c>
     </row>
-    <row r="184" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A184" t="s">
         <v>14</v>
       </c>
       <c r="C184" s="1">
-        <v>46262.00060185185</v>
+        <v>46262.000601851847</v>
       </c>
       <c r="D184" t="s">
         <v>246</v>
@@ -5314,12 +5340,12 @@
         <v>2955616</v>
       </c>
     </row>
-    <row r="185" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A185" t="s">
         <v>14</v>
       </c>
       <c r="C185" s="1">
-        <v>46266.00060185185</v>
+        <v>46266.000601851847</v>
       </c>
       <c r="D185" t="s">
         <v>247</v>
@@ -5334,12 +5360,12 @@
         <v>1207890</v>
       </c>
     </row>
-    <row r="186" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A186" t="s">
         <v>14</v>
       </c>
       <c r="C186" s="1">
-        <v>46266.00060185185</v>
+        <v>46266.000601851847</v>
       </c>
       <c r="D186" t="s">
         <v>248</v>
@@ -5354,12 +5380,12 @@
         <v>7137643</v>
       </c>
     </row>
-    <row r="187" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A187" t="s">
         <v>14</v>
       </c>
       <c r="C187" s="1">
-        <v>46273.00060185185</v>
+        <v>46273.000601851847</v>
       </c>
       <c r="D187" t="s">
         <v>249</v>
@@ -5374,12 +5400,12 @@
         <v>213339</v>
       </c>
     </row>
-    <row r="188" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A188" t="s">
         <v>14</v>
       </c>
       <c r="C188" s="1">
-        <v>46277.00060185185</v>
+        <v>46277.000601851847</v>
       </c>
       <c r="D188" t="s">
         <v>250</v>
@@ -5394,12 +5420,12 @@
         <v>3637191</v>
       </c>
     </row>
-    <row r="189" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A189" t="s">
         <v>14</v>
       </c>
       <c r="C189" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D189" t="s">
         <v>251</v>
@@ -5414,12 +5440,12 @@
         <v>3139397</v>
       </c>
     </row>
-    <row r="190" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A190" t="s">
         <v>14</v>
       </c>
       <c r="C190" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D190" t="s">
         <v>252</v>
@@ -5434,12 +5460,12 @@
         <v>16697534</v>
       </c>
     </row>
-    <row r="191" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A191" t="s">
         <v>14</v>
       </c>
       <c r="C191" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D191" t="s">
         <v>253</v>
@@ -5454,12 +5480,12 @@
         <v>3186630</v>
       </c>
     </row>
-    <row r="192" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A192" t="s">
         <v>14</v>
       </c>
       <c r="C192" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D192" t="s">
         <v>254</v>
@@ -5474,12 +5500,12 @@
         <v>8726027</v>
       </c>
     </row>
-    <row r="193" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A193" t="s">
         <v>14</v>
       </c>
       <c r="C193" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D193" t="s">
         <v>255</v>
@@ -5494,12 +5520,12 @@
         <v>8391945</v>
       </c>
     </row>
-    <row r="194" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A194" t="s">
         <v>14</v>
       </c>
       <c r="C194" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D194" t="s">
         <v>256</v>
@@ -5514,12 +5540,12 @@
         <v>7613869</v>
       </c>
     </row>
-    <row r="195" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A195" t="s">
         <v>14</v>
       </c>
       <c r="C195" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D195" t="s">
         <v>257</v>
@@ -5534,12 +5560,12 @@
         <v>3812681</v>
       </c>
     </row>
-    <row r="196" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A196" t="s">
         <v>14</v>
       </c>
       <c r="C196" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D196" t="s">
         <v>258</v>
@@ -5554,12 +5580,12 @@
         <v>2631452</v>
       </c>
     </row>
-    <row r="197" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A197" t="s">
         <v>14</v>
       </c>
       <c r="C197" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D197" t="s">
         <v>259</v>
@@ -5574,12 +5600,12 @@
         <v>6901008</v>
       </c>
     </row>
-    <row r="198" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A198" t="s">
         <v>14</v>
       </c>
       <c r="C198" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D198" t="s">
         <v>260</v>
@@ -5594,12 +5620,12 @@
         <v>1657008</v>
       </c>
     </row>
-    <row r="199" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A199" t="s">
         <v>14</v>
       </c>
       <c r="C199" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D199" t="s">
         <v>261</v>
@@ -5614,12 +5640,12 @@
         <v>4389534</v>
       </c>
     </row>
-    <row r="200" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A200" t="s">
         <v>14</v>
       </c>
       <c r="C200" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D200" t="s">
         <v>262</v>
@@ -5634,12 +5660,12 @@
         <v>2926356</v>
       </c>
     </row>
-    <row r="201" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A201" t="s">
         <v>14</v>
       </c>
       <c r="C201" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D201" t="s">
         <v>261</v>
@@ -5654,12 +5680,12 @@
         <v>4389534</v>
       </c>
     </row>
-    <row r="202" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A202" t="s">
         <v>14</v>
       </c>
       <c r="C202" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D202" t="s">
         <v>263</v>
@@ -5674,12 +5700,12 @@
         <v>1463178</v>
       </c>
     </row>
-    <row r="203" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A203" t="s">
         <v>14</v>
       </c>
       <c r="C203" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D203" t="s">
         <v>264</v>
@@ -5694,12 +5720,12 @@
         <v>3520499</v>
       </c>
     </row>
-    <row r="204" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A204" t="s">
         <v>14</v>
       </c>
       <c r="C204" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D204" t="s">
         <v>265</v>
@@ -5714,12 +5740,12 @@
         <v>708878</v>
       </c>
     </row>
-    <row r="205" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A205" t="s">
         <v>14</v>
       </c>
       <c r="C205" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D205" t="s">
         <v>266</v>
@@ -5734,12 +5760,12 @@
         <v>1269386</v>
       </c>
     </row>
-    <row r="206" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A206" t="s">
         <v>14</v>
       </c>
       <c r="C206" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D206" t="s">
         <v>267</v>
@@ -5754,12 +5780,12 @@
         <v>123770</v>
       </c>
     </row>
-    <row r="207" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A207" t="s">
         <v>14</v>
       </c>
       <c r="C207" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D207" t="s">
         <v>268</v>
@@ -5774,12 +5800,12 @@
         <v>20543561</v>
       </c>
     </row>
-    <row r="208" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A208" t="s">
         <v>14</v>
       </c>
       <c r="C208" s="1">
-        <v>46280.00060185185</v>
+        <v>46280.000601851847</v>
       </c>
       <c r="D208" t="s">
         <v>269</v>
@@ -5794,12 +5820,12 @@
         <v>9244602</v>
       </c>
     </row>
-    <row r="209" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A209" t="s">
         <v>14</v>
       </c>
       <c r="C209" s="1">
-        <v>46281.00060185185</v>
+        <v>46281.000601851847</v>
       </c>
       <c r="D209" t="s">
         <v>270</v>
@@ -5814,12 +5840,12 @@
         <v>5996164</v>
       </c>
     </row>
-    <row r="210" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A210" t="s">
         <v>14</v>
       </c>
       <c r="C210" s="1">
-        <v>46282.00060185185</v>
+        <v>46282.000601851847</v>
       </c>
       <c r="D210" t="s">
         <v>271</v>
@@ -5834,12 +5860,12 @@
         <v>3873726</v>
       </c>
     </row>
-    <row r="211" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A211" t="s">
         <v>14</v>
       </c>
       <c r="C211" s="1">
-        <v>46282.00060185185</v>
+        <v>46282.000601851847</v>
       </c>
       <c r="D211" t="s">
         <v>272</v>
@@ -5854,12 +5880,12 @@
         <v>14302465</v>
       </c>
     </row>
-    <row r="212" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A212" t="s">
         <v>14</v>
       </c>
       <c r="C212" s="1">
-        <v>46287.00060185185</v>
+        <v>46287.000601851847</v>
       </c>
       <c r="D212" t="s">
         <v>273</v>
@@ -5874,12 +5900,12 @@
         <v>10308986</v>
       </c>
     </row>
-    <row r="213" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A213" t="s">
         <v>14</v>
       </c>
       <c r="C213" s="1">
-        <v>46294.00060185185</v>
+        <v>46294.000601851847</v>
       </c>
       <c r="D213" t="s">
         <v>274</v>
@@ -5894,12 +5920,12 @@
         <v>19807403</v>
       </c>
     </row>
-    <row r="214" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A214" t="s">
         <v>14</v>
       </c>
       <c r="C214" s="1">
-        <v>46294.00060185185</v>
+        <v>46294.000601851847</v>
       </c>
       <c r="D214" t="s">
         <v>275</v>
@@ -5914,12 +5940,12 @@
         <v>2621326</v>
       </c>
     </row>
-    <row r="215" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A215" t="s">
         <v>14</v>
       </c>
       <c r="C215" s="1">
-        <v>46294.00060185185</v>
+        <v>46294.000601851847</v>
       </c>
       <c r="D215" t="s">
         <v>276</v>
@@ -5934,12 +5960,12 @@
         <v>957517</v>
       </c>
     </row>
-    <row r="216" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A216" t="s">
         <v>14</v>
       </c>
       <c r="C216" s="1">
-        <v>46294.00060185185</v>
+        <v>46294.000601851847</v>
       </c>
       <c r="D216" t="s">
         <v>277</v>
@@ -5954,12 +5980,12 @@
         <v>8466312</v>
       </c>
     </row>
-    <row r="217" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A217" t="s">
         <v>14</v>
       </c>
       <c r="C217" s="1">
-        <v>46294.00060185185</v>
+        <v>46294.000601851847</v>
       </c>
       <c r="D217" t="s">
         <v>278</v>
@@ -5974,12 +6000,12 @@
         <v>1199587</v>
       </c>
     </row>
-    <row r="218" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A218" t="s">
         <v>14</v>
       </c>
       <c r="C218" s="1">
-        <v>46294.00060185185</v>
+        <v>46294.000601851847</v>
       </c>
       <c r="D218" t="s">
         <v>279</v>
@@ -5994,12 +6020,12 @@
         <v>2955616</v>
       </c>
     </row>
-    <row r="219" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A219" t="s">
         <v>14</v>
       </c>
       <c r="C219" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D219" t="s">
         <v>280</v>
@@ -6014,12 +6040,12 @@
         <v>6907397</v>
       </c>
     </row>
-    <row r="220" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A220" t="s">
         <v>14</v>
       </c>
       <c r="C220" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D220" t="s">
         <v>281</v>
@@ -6034,12 +6060,12 @@
         <v>2359371</v>
       </c>
     </row>
-    <row r="221" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A221" t="s">
         <v>14</v>
       </c>
       <c r="C221" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D221" t="s">
         <v>282</v>
@@ -6054,12 +6080,12 @@
         <v>2298874</v>
       </c>
     </row>
-    <row r="222" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A222" t="s">
         <v>14</v>
       </c>
       <c r="C222" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D222" t="s">
         <v>283</v>
@@ -6074,12 +6100,12 @@
         <v>854071</v>
       </c>
     </row>
-    <row r="223" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A223" t="s">
         <v>14</v>
       </c>
       <c r="C223" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D223" t="s">
         <v>284</v>
@@ -6094,12 +6120,12 @@
         <v>907450</v>
       </c>
     </row>
-    <row r="224" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A224" t="s">
         <v>14</v>
       </c>
       <c r="C224" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D224" t="s">
         <v>285</v>
@@ -6114,12 +6140,12 @@
         <v>626645</v>
       </c>
     </row>
-    <row r="225" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A225" t="s">
         <v>14</v>
       </c>
       <c r="C225" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D225" t="s">
         <v>286</v>
@@ -6134,12 +6160,12 @@
         <v>569380</v>
       </c>
     </row>
-    <row r="226" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A226" t="s">
         <v>14</v>
       </c>
       <c r="C226" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D226" t="s">
         <v>287</v>
@@ -6154,12 +6180,12 @@
         <v>241986</v>
       </c>
     </row>
-    <row r="227" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A227" t="s">
         <v>14</v>
       </c>
       <c r="C227" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D227" t="s">
         <v>288</v>
@@ -6174,12 +6200,12 @@
         <v>5316592</v>
       </c>
     </row>
-    <row r="228" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A228" t="s">
         <v>14</v>
       </c>
       <c r="C228" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D228" t="s">
         <v>288</v>
@@ -6194,12 +6220,12 @@
         <v>5316592</v>
       </c>
     </row>
-    <row r="229" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A229" t="s">
         <v>14</v>
       </c>
       <c r="C229" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D229" t="s">
         <v>289</v>
@@ -6214,12 +6240,12 @@
         <v>9537127</v>
       </c>
     </row>
-    <row r="230" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A230" t="s">
         <v>14</v>
       </c>
       <c r="C230" s="1">
-        <v>46295.00060185185</v>
+        <v>46295.000601851847</v>
       </c>
       <c r="D230" t="s">
         <v>290</v>
@@ -6234,12 +6260,12 @@
         <v>3531567</v>
       </c>
     </row>
-    <row r="231" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A231" t="s">
         <v>14</v>
       </c>
       <c r="C231" s="1">
-        <v>46296.00060185185</v>
+        <v>46296.000601851847</v>
       </c>
       <c r="D231" t="s">
         <v>291</v>
@@ -6254,12 +6280,12 @@
         <v>1329041</v>
       </c>
     </row>
-    <row r="232" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A232" t="s">
         <v>14</v>
       </c>
       <c r="C232" s="1">
-        <v>46296.00060185185</v>
+        <v>46296.000601851847</v>
       </c>
       <c r="D232" t="s">
         <v>292</v>
@@ -6274,12 +6300,12 @@
         <v>13906</v>
       </c>
     </row>
-    <row r="233" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A233" t="s">
         <v>14</v>
       </c>
       <c r="C233" s="1">
-        <v>46308.00060185185</v>
+        <v>46308.000601851847</v>
       </c>
       <c r="D233" t="s">
         <v>293</v>
@@ -6294,12 +6320,12 @@
         <v>3519863</v>
       </c>
     </row>
-    <row r="234" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A234" t="s">
         <v>14</v>
       </c>
       <c r="C234" s="1">
-        <v>46310.00060185185</v>
+        <v>46310.000601851847</v>
       </c>
       <c r="D234" t="s">
         <v>294</v>
@@ -6314,12 +6340,12 @@
         <v>3529315</v>
       </c>
     </row>
-    <row r="235" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A235" t="s">
         <v>14</v>
       </c>
       <c r="C235" s="1">
-        <v>46310.00060185185</v>
+        <v>46310.000601851847</v>
       </c>
       <c r="D235" t="s">
         <v>295</v>
@@ -6334,12 +6360,12 @@
         <v>16076712</v>
       </c>
     </row>
-    <row r="236" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A236" t="s">
         <v>14</v>
       </c>
       <c r="C236" s="1">
-        <v>46310.00060185185</v>
+        <v>46310.000601851847</v>
       </c>
       <c r="D236" t="s">
         <v>296</v>
@@ -6354,12 +6380,12 @@
         <v>3067397</v>
       </c>
     </row>
-    <row r="237" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A237" t="s">
         <v>14</v>
       </c>
       <c r="C237" s="1">
-        <v>46311.00060185185</v>
+        <v>46311.000601851847</v>
       </c>
       <c r="D237" t="s">
         <v>297</v>
@@ -6374,12 +6400,12 @@
         <v>5802739</v>
       </c>
     </row>
-    <row r="238" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A238" t="s">
         <v>14</v>
       </c>
       <c r="C238" s="1">
-        <v>46312.00060185185</v>
+        <v>46312.000601851847</v>
       </c>
       <c r="D238" t="s">
         <v>298</v>
@@ -6394,12 +6420,12 @@
         <v>13841095</v>
       </c>
     </row>
-    <row r="239" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A239" t="s">
         <v>14</v>
       </c>
       <c r="C239" s="1">
-        <v>46312.00060185185</v>
+        <v>46312.000601851847</v>
       </c>
       <c r="D239" t="s">
         <v>299</v>
@@ -6414,12 +6440,12 @@
         <v>3748767</v>
       </c>
     </row>
-    <row r="240" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A240" t="s">
         <v>14</v>
       </c>
       <c r="C240" s="1">
-        <v>46316.00060185185</v>
+        <v>46316.000601851847</v>
       </c>
       <c r="D240" t="s">
         <v>300</v>
@@ -6434,12 +6460,12 @@
         <v>9976438</v>
       </c>
     </row>
-    <row r="241" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A241" t="s">
         <v>14</v>
       </c>
       <c r="C241" s="1">
-        <v>46322.00060185185</v>
+        <v>46322.000601851847</v>
       </c>
       <c r="D241" t="s">
         <v>301</v>
@@ -6454,12 +6480,12 @@
         <v>19168454</v>
       </c>
     </row>
-    <row r="242" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A242" t="s">
         <v>14</v>
       </c>
       <c r="C242" s="1">
-        <v>46322.00060185185</v>
+        <v>46322.000601851847</v>
       </c>
       <c r="D242" t="s">
         <v>302</v>
@@ -6474,12 +6500,12 @@
         <v>2520328</v>
       </c>
     </row>
-    <row r="243" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A243" t="s">
         <v>14</v>
       </c>
       <c r="C243" s="1">
-        <v>46322.00060185185</v>
+        <v>46322.000601851847</v>
       </c>
       <c r="D243" t="s">
         <v>303</v>
@@ -6494,12 +6520,12 @@
         <v>945123</v>
       </c>
     </row>
-    <row r="244" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A244" t="s">
         <v>14</v>
       </c>
       <c r="C244" s="1">
-        <v>46323.00060185185</v>
+        <v>46323.000601851847</v>
       </c>
       <c r="D244" t="s">
         <v>304</v>
@@ -6514,12 +6540,12 @@
         <v>8193205</v>
       </c>
     </row>
-    <row r="245" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A245" t="s">
         <v>14</v>
       </c>
       <c r="C245" s="1">
-        <v>46323.00060185185</v>
+        <v>46323.000601851847</v>
       </c>
       <c r="D245" t="s">
         <v>305</v>
@@ -6534,12 +6560,12 @@
         <v>1193835</v>
       </c>
     </row>
-    <row r="246" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A246" t="s">
         <v>14</v>
       </c>
       <c r="C246" s="1">
-        <v>46323.00060185185</v>
+        <v>46323.000601851847</v>
       </c>
       <c r="D246" t="s">
         <v>306</v>
@@ -6554,12 +6580,12 @@
         <v>2860273</v>
       </c>
     </row>
-    <row r="247" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A247" t="s">
         <v>14</v>
       </c>
       <c r="C247" s="1">
-        <v>46326.00060185185</v>
+        <v>46326.000601851847</v>
       </c>
       <c r="D247" t="s">
         <v>307</v>
@@ -6574,12 +6600,12 @@
         <v>7137643</v>
       </c>
     </row>
-    <row r="248" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A248" t="s">
         <v>14</v>
       </c>
       <c r="C248" s="1">
-        <v>46329.00060185185</v>
+        <v>46329.000601851847</v>
       </c>
       <c r="D248" t="s">
         <v>308</v>
@@ -6594,12 +6620,12 @@
         <v>1373342</v>
       </c>
     </row>
-    <row r="249" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A249" t="s">
         <v>14</v>
       </c>
       <c r="C249" s="1">
-        <v>46332.00060185185</v>
+        <v>46332.000601851847</v>
       </c>
       <c r="D249" t="s">
         <v>309</v>
@@ -6614,12 +6640,12 @@
         <v>664573</v>
       </c>
     </row>
-    <row r="250" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A250" t="s">
         <v>14</v>
       </c>
       <c r="C250" s="1">
-        <v>46338.00060185185</v>
+        <v>46338.000601851847</v>
       </c>
       <c r="D250" t="s">
         <v>310</v>
@@ -6634,12 +6660,12 @@
         <v>3637191</v>
       </c>
     </row>
-    <row r="251" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A251" t="s">
         <v>14</v>
       </c>
       <c r="C251" s="1">
-        <v>46343.00060185185</v>
+        <v>46343.000601851847</v>
       </c>
       <c r="D251" t="s">
         <v>311</v>
@@ -6654,12 +6680,12 @@
         <v>3646958</v>
       </c>
     </row>
-    <row r="252" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A252" t="s">
         <v>14</v>
       </c>
       <c r="C252" s="1">
-        <v>46343.00060185185</v>
+        <v>46343.000601851847</v>
       </c>
       <c r="D252" t="s">
         <v>312</v>
@@ -6674,12 +6700,12 @@
         <v>3873726</v>
       </c>
     </row>
-    <row r="253" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A253" t="s">
         <v>14</v>
       </c>
       <c r="C253" s="1">
-        <v>46343.00060185185</v>
+        <v>46343.000601851847</v>
       </c>
       <c r="D253" t="s">
         <v>313</v>
@@ -6694,12 +6720,12 @@
         <v>16612602</v>
       </c>
     </row>
-    <row r="254" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A254" t="s">
         <v>14</v>
       </c>
       <c r="C254" s="1">
-        <v>46343.00060185185</v>
+        <v>46343.000601851847</v>
       </c>
       <c r="D254" t="s">
         <v>314</v>
@@ -6714,12 +6740,12 @@
         <v>3169643</v>
       </c>
     </row>
-    <row r="255" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A255" t="s">
         <v>14</v>
       </c>
       <c r="C255" s="1">
-        <v>46343.00060185185</v>
+        <v>46343.000601851847</v>
       </c>
       <c r="D255" t="s">
         <v>315</v>
@@ -6734,12 +6760,12 @@
         <v>6047123</v>
       </c>
     </row>
-    <row r="256" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A256" t="s">
         <v>14</v>
       </c>
       <c r="C256" s="1">
-        <v>46343.00060185185</v>
+        <v>46343.000601851847</v>
       </c>
       <c r="D256" t="s">
         <v>316</v>
@@ -6754,12 +6780,12 @@
         <v>12569863</v>
       </c>
     </row>
-    <row r="257" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A257" t="s">
         <v>14</v>
       </c>
       <c r="C257" s="1">
-        <v>46347.00060185185</v>
+        <v>46347.000601851847</v>
       </c>
       <c r="D257" t="s">
         <v>317</v>
@@ -6774,12 +6800,12 @@
         <v>10359945</v>
       </c>
     </row>
-    <row r="258" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A258" t="s">
         <v>14</v>
       </c>
       <c r="C258" s="1">
-        <v>46353.00060185185</v>
+        <v>46353.000601851847</v>
       </c>
       <c r="D258" t="s">
         <v>318</v>
@@ -6794,12 +6820,12 @@
         <v>19807403</v>
       </c>
     </row>
-    <row r="259" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A259" t="s">
         <v>14</v>
       </c>
       <c r="C259" s="1">
-        <v>46353.00060185185</v>
+        <v>46353.000601851847</v>
       </c>
       <c r="D259" t="s">
         <v>319</v>
@@ -6814,12 +6840,12 @@
         <v>2604339</v>
       </c>
     </row>
-    <row r="260" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A260" t="s">
         <v>14</v>
       </c>
       <c r="C260" s="1">
-        <v>46353.00060185185</v>
+        <v>46353.000601851847</v>
       </c>
       <c r="D260" t="s">
         <v>320</v>
@@ -6834,12 +6860,12 @@
         <v>976627</v>
       </c>
     </row>
-    <row r="261" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A261" t="s">
         <v>14</v>
       </c>
       <c r="C261" s="1">
-        <v>46354.00060185185</v>
+        <v>46354.000601851847</v>
       </c>
       <c r="D261" t="s">
         <v>321</v>
@@ -6854,12 +6880,12 @@
         <v>8535106</v>
       </c>
     </row>
-    <row r="262" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A262" t="s">
         <v>14</v>
       </c>
       <c r="C262" s="1">
-        <v>46354.00060185185</v>
+        <v>46354.000601851847</v>
       </c>
       <c r="D262" t="s">
         <v>322</v>
@@ -6874,12 +6900,12 @@
         <v>1233630</v>
       </c>
     </row>
-    <row r="263" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A263" t="s">
         <v>14</v>
       </c>
       <c r="C263" s="1">
-        <v>46354.00060185185</v>
+        <v>46354.000601851847</v>
       </c>
       <c r="D263" t="s">
         <v>323</v>
@@ -6894,12 +6920,12 @@
         <v>2955616</v>
       </c>
     </row>
-    <row r="264" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A264" t="s">
         <v>14</v>
       </c>
       <c r="C264" s="1">
-        <v>46357.00060185185</v>
+        <v>46357.000601851847</v>
       </c>
       <c r="D264" t="s">
         <v>324</v>
@@ -6914,12 +6940,12 @@
         <v>1329041</v>
       </c>
     </row>
-    <row r="265" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A265" t="s">
         <v>14</v>
       </c>
       <c r="C265" s="1">
-        <v>46357.00060185185</v>
+        <v>46357.000601851847</v>
       </c>
       <c r="D265" t="s">
         <v>325</v>
@@ -6934,12 +6960,12 @@
         <v>6907397</v>
       </c>
     </row>
-    <row r="266" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A266" t="s">
         <v>14</v>
       </c>
       <c r="C266" s="1">
-        <v>46364.00060185185</v>
+        <v>46364.000601851847</v>
       </c>
       <c r="D266" t="s">
         <v>326</v>
@@ -6954,12 +6980,12 @@
         <v>252765</v>
       </c>
     </row>
-    <row r="267" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A267" t="s">
         <v>14</v>
       </c>
       <c r="C267" s="1">
-        <v>46368.00060185185</v>
+        <v>46368.000601851847</v>
       </c>
       <c r="D267" t="s">
         <v>327</v>
@@ -6974,12 +7000,12 @@
         <v>3519863</v>
       </c>
     </row>
-    <row r="268" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A268" t="s">
         <v>14</v>
       </c>
       <c r="C268" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D268" t="s">
         <v>328</v>
@@ -6994,12 +7020,12 @@
         <v>3529315</v>
       </c>
     </row>
-    <row r="269" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A269" t="s">
         <v>14</v>
       </c>
       <c r="C269" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D269" t="s">
         <v>329</v>
@@ -7014,12 +7040,12 @@
         <v>16076712</v>
       </c>
     </row>
-    <row r="270" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A270" t="s">
         <v>14</v>
       </c>
       <c r="C270" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D270" t="s">
         <v>330</v>
@@ -7034,12 +7060,12 @@
         <v>3067397</v>
       </c>
     </row>
-    <row r="271" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A271" t="s">
         <v>14</v>
       </c>
       <c r="C271" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D271" t="s">
         <v>331</v>
@@ -7054,12 +7080,12 @@
         <v>8528766</v>
       </c>
     </row>
-    <row r="272" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A272" t="s">
         <v>14</v>
       </c>
       <c r="C272" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D272" t="s">
         <v>332</v>
@@ -7074,12 +7100,12 @@
         <v>8196657</v>
       </c>
     </row>
-    <row r="273" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A273" t="s">
         <v>14</v>
       </c>
       <c r="C273" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D273" t="s">
         <v>333</v>
@@ -7094,12 +7120,12 @@
         <v>7531110</v>
       </c>
     </row>
-    <row r="274" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A274" t="s">
         <v>14</v>
       </c>
       <c r="C274" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D274" t="s">
         <v>334</v>
@@ -7114,12 +7140,12 @@
         <v>3771239</v>
       </c>
     </row>
-    <row r="275" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A275" t="s">
         <v>14</v>
       </c>
       <c r="C275" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D275" t="s">
         <v>335</v>
@@ -7134,12 +7160,12 @@
         <v>2602849</v>
       </c>
     </row>
-    <row r="276" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A276" t="s">
         <v>14</v>
       </c>
       <c r="C276" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D276" t="s">
         <v>336</v>
@@ -7154,12 +7180,12 @@
         <v>6825997</v>
       </c>
     </row>
-    <row r="277" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A277" t="s">
         <v>14</v>
       </c>
       <c r="C277" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D277" t="s">
         <v>337</v>
@@ -7174,12 +7200,12 @@
         <v>1638997</v>
       </c>
     </row>
-    <row r="278" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A278" t="s">
         <v>14</v>
       </c>
       <c r="C278" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D278" t="s">
         <v>338</v>
@@ -7194,12 +7220,12 @@
         <v>4341821</v>
       </c>
     </row>
-    <row r="279" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A279" t="s">
         <v>14</v>
       </c>
       <c r="C279" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D279" t="s">
         <v>339</v>
@@ -7214,12 +7240,12 @@
         <v>2894547</v>
       </c>
     </row>
-    <row r="280" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A280" t="s">
         <v>14</v>
       </c>
       <c r="C280" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D280" t="s">
         <v>338</v>
@@ -7234,12 +7260,12 @@
         <v>4341821</v>
       </c>
     </row>
-    <row r="281" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A281" t="s">
         <v>14</v>
       </c>
       <c r="C281" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D281" t="s">
         <v>340</v>
@@ -7254,12 +7280,12 @@
         <v>1447273</v>
       </c>
     </row>
-    <row r="282" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A282" t="s">
         <v>14</v>
       </c>
       <c r="C282" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D282" t="s">
         <v>341</v>
@@ -7274,12 +7300,12 @@
         <v>3482233</v>
       </c>
     </row>
-    <row r="283" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A283" t="s">
         <v>14</v>
       </c>
       <c r="C283" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D283" t="s">
         <v>342</v>
@@ -7294,12 +7320,12 @@
         <v>701173</v>
       </c>
     </row>
-    <row r="284" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A284" t="s">
         <v>14</v>
       </c>
       <c r="C284" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D284" t="s">
         <v>343</v>
@@ -7314,12 +7340,12 @@
         <v>2179512</v>
       </c>
     </row>
-    <row r="285" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A285" t="s">
         <v>14</v>
       </c>
       <c r="C285" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D285" t="s">
         <v>344</v>
@@ -7334,12 +7360,12 @@
         <v>625730</v>
       </c>
     </row>
-    <row r="286" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A286" t="s">
         <v>14</v>
       </c>
       <c r="C286" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D286" t="s">
         <v>345</v>
@@ -7354,12 +7380,12 @@
         <v>440284</v>
       </c>
     </row>
-    <row r="287" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A287" t="s">
         <v>14</v>
       </c>
       <c r="C287" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D287" t="s">
         <v>346</v>
@@ -7374,12 +7400,12 @@
         <v>20149040</v>
       </c>
     </row>
-    <row r="288" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A288" t="s">
         <v>14</v>
       </c>
       <c r="C288" s="1">
-        <v>46371.00060185185</v>
+        <v>46371.000601851847</v>
       </c>
       <c r="D288" t="s">
         <v>347</v>
@@ -7394,12 +7420,12 @@
         <v>9067068</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A289" t="s">
         <v>14</v>
       </c>
       <c r="C289" s="1">
-        <v>46372.00060185185</v>
+        <v>46372.000601851847</v>
       </c>
       <c r="D289" t="s">
         <v>348</v>
@@ -7414,12 +7440,12 @@
         <v>5852054</v>
       </c>
     </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A290" t="s">
         <v>14</v>
       </c>
       <c r="C290" s="1">
-        <v>46373.00060185185</v>
+        <v>46373.000601851847</v>
       </c>
       <c r="D290" t="s">
         <v>349</v>
@@ -7434,12 +7460,12 @@
         <v>3748767</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A291" t="s">
         <v>14</v>
       </c>
       <c r="C291" s="1">
-        <v>46373.00060185185</v>
+        <v>46373.000601851847</v>
       </c>
       <c r="D291" t="s">
         <v>350</v>
@@ -7454,12 +7480,12 @@
         <v>12164383</v>
       </c>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A292" t="s">
         <v>14</v>
       </c>
       <c r="C292" s="1">
-        <v>46378.00060185185</v>
+        <v>46378.000601851847</v>
       </c>
       <c r="D292" t="s">
         <v>351</v>
@@ -7474,12 +7500,12 @@
         <v>10025753</v>
       </c>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A293" t="s">
         <v>14</v>
       </c>
       <c r="C293" s="1">
-        <v>46385.00060185185</v>
+        <v>46385.000601851847</v>
       </c>
       <c r="D293" t="s">
         <v>352</v>
@@ -7494,12 +7520,12 @@
         <v>19168454</v>
       </c>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A294" t="s">
         <v>14</v>
       </c>
       <c r="C294" s="1">
-        <v>46385.00060185185</v>
+        <v>46385.000601851847</v>
       </c>
       <c r="D294" t="s">
         <v>353</v>
@@ -7514,12 +7540,12 @@
         <v>2520328</v>
       </c>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A295" t="s">
         <v>14</v>
       </c>
       <c r="C295" s="1">
-        <v>46385.00060185185</v>
+        <v>46385.000601851847</v>
       </c>
       <c r="D295" t="s">
         <v>354</v>
@@ -7534,12 +7560,12 @@
         <v>945123</v>
       </c>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A296" t="s">
         <v>14</v>
       </c>
       <c r="C296" s="1">
-        <v>46385.00060185185</v>
+        <v>46385.000601851847</v>
       </c>
       <c r="D296" t="s">
         <v>355</v>
@@ -7554,12 +7580,12 @@
         <v>8259780</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A297" t="s">
         <v>14</v>
       </c>
       <c r="C297" s="1">
-        <v>46385.00060185185</v>
+        <v>46385.000601851847</v>
       </c>
       <c r="D297" t="s">
         <v>356</v>
@@ -7574,12 +7600,12 @@
         <v>1193835</v>
       </c>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A298" t="s">
         <v>14</v>
       </c>
       <c r="C298" s="1">
-        <v>46385.00060185185</v>
+        <v>46385.000601851847</v>
       </c>
       <c r="D298" t="s">
         <v>357</v>
@@ -7594,12 +7620,12 @@
         <v>2860273</v>
       </c>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A299" t="s">
         <v>14</v>
       </c>
       <c r="C299" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D299" t="s">
         <v>358</v>
@@ -7614,12 +7640,12 @@
         <v>7137643</v>
       </c>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A300" t="s">
         <v>14</v>
       </c>
       <c r="C300" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D300" t="s">
         <v>359</v>
@@ -7634,12 +7660,12 @@
         <v>2405871</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A301" t="s">
         <v>14</v>
       </c>
       <c r="C301" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D301" t="s">
         <v>360</v>
@@ -7654,12 +7680,12 @@
         <v>2344183</v>
       </c>
     </row>
-    <row r="302" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A302" t="s">
         <v>14</v>
       </c>
       <c r="C302" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D302" t="s">
         <v>361</v>
@@ -7674,12 +7700,12 @@
         <v>870903</v>
       </c>
     </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A303" t="s">
         <v>14</v>
       </c>
       <c r="C303" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D303" t="s">
         <v>362</v>
@@ -7694,12 +7720,12 @@
         <v>925334</v>
       </c>
     </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A304" t="s">
         <v>14</v>
       </c>
       <c r="C304" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D304" t="s">
         <v>363</v>
@@ -7714,12 +7740,12 @@
         <v>653177</v>
       </c>
     </row>
-    <row r="305" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A305" t="s">
         <v>14</v>
       </c>
       <c r="C305" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D305" t="s">
         <v>364</v>
@@ -7734,12 +7760,12 @@
         <v>580601</v>
       </c>
     </row>
-    <row r="306" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A306" t="s">
         <v>14</v>
       </c>
       <c r="C306" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D306" t="s">
         <v>365</v>
@@ -7754,12 +7780,12 @@
         <v>246755</v>
       </c>
     </row>
-    <row r="307" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A307" t="s">
         <v>14</v>
       </c>
       <c r="C307" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D307" t="s">
         <v>366</v>
@@ -7774,12 +7800,12 @@
         <v>5421377</v>
       </c>
     </row>
-    <row r="308" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A308" t="s">
         <v>14</v>
       </c>
       <c r="C308" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D308" t="s">
         <v>366</v>
@@ -7794,12 +7820,12 @@
         <v>5421377</v>
       </c>
     </row>
-    <row r="309" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A309" t="s">
         <v>14</v>
       </c>
       <c r="C309" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D309" t="s">
         <v>367</v>
@@ -7814,12 +7840,12 @@
         <v>9725095</v>
       </c>
     </row>
-    <row r="310" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A310" t="s">
         <v>14</v>
       </c>
       <c r="C310" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D310" t="s">
         <v>368</v>
@@ -7834,12 +7860,12 @@
         <v>11847924</v>
       </c>
     </row>
-    <row r="311" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A311" t="s">
         <v>14</v>
       </c>
       <c r="C311" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D311" t="s">
         <v>369</v>
@@ -7848,12 +7874,12 @@
         <v>-59756037</v>
       </c>
     </row>
-    <row r="312" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A312" t="s">
         <v>14</v>
       </c>
       <c r="C312" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D312" t="s">
         <v>370</v>
@@ -7862,12 +7888,12 @@
         <v>55567664</v>
       </c>
     </row>
-    <row r="313" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A313" t="s">
         <v>14</v>
       </c>
       <c r="C313" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D313" t="s">
         <v>371</v>
@@ -7876,12 +7902,12 @@
         <v>775582</v>
       </c>
     </row>
-    <row r="314" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A314" t="s">
         <v>14</v>
       </c>
       <c r="C314" s="1">
-        <v>46387.00060185185</v>
+        <v>46387.000601851847</v>
       </c>
       <c r="D314" t="s">
         <v>372</v>
@@ -7891,7 +7917,8 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>